<commit_message>
updated with latest data
</commit_message>
<xml_diff>
--- a/data/metadata.xlsx
+++ b/data/metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://psrcwa-my.sharepoint.com/personal/chelmann_psrc_org/Documents/coding/centers-monitoring/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{6E65EA87-A5EF-4E28-BE4A-4C8238B7EF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47ECD86C-984B-40D8-9120-BE61CD48C5E8}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{6E65EA87-A5EF-4E28-BE4A-4C8238B7EF95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AAB61F0-493C-4E95-A066-0BA63AC8A88B}"/>
   <bookViews>
-    <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{74B535C6-8259-44B5-AC9A-6ED9B66D2469}"/>
+    <workbookView xWindow="34440" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{74B535C6-8259-44B5-AC9A-6ED9B66D2469}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Notes" sheetId="1" r:id="rId1"/>
@@ -81,10 +81,10 @@
 Employment summaries derive from the Quarterly Census of Employment and Wages (QCEW), administrative records employers report, by law, to the Washington State Employment Security Department (ESD).  To provide more accurate workplace reporting, PSRC gathers supplemental data from the Boeing Company, the Office of Washington Superintendent of Public Instruction (OSPI), and governmental units throughout the central Puget Sound region. The unit of measurement is jobs, rather than working persons or proportional full-time employment (FTE) equivalents.  Part-time and temporary positions are included.</t>
   </si>
   <si>
-    <t>Total population and housing units are generated using the Office of Financial Management's Small area Estimate Program (SAEP) block data. This data is available by Census block from 2010 through 2022. The blocks are parcelized by PSRC using its base-year model parcel inputs. The parcel centroids that are contained within a given center are aggregated for that center.</t>
+    <t>Data Update Date:</t>
   </si>
   <si>
-    <t>Data Update Date:</t>
+    <t>Total population and housing units are generated using the Office of Financial Management's Small area Estimate Program (SAEP) block data. This data is available by Census block from 2010 through 2025. The blocks are parcelized by PSRC using its base-year model parcel inputs. The parcel centroids that are contained within a given center are aggregated for that center.</t>
   </si>
 </sst>
 </file>
@@ -165,6 +165,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -179,15 +188,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -531,70 +531,70 @@
     </row>
     <row r="2" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3"/>
+    </row>
+    <row r="3" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9"/>
+    <row r="4" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
+      <c r="A4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
+      <c r="A5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9"/>
-    <row r="4" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A4" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A5" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
     </row>
     <row r="8" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
     </row>
     <row r="9" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
     </row>
     <row r="10" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
     </row>
     <row r="11" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
       <c r="A11" s="4"/>
@@ -605,450 +605,450 @@
       <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.9">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
     </row>
     <row r="13" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
     </row>
     <row r="14" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
     </row>
     <row r="15" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
     </row>
     <row r="16" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
     </row>
     <row r="17" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
     </row>
     <row r="18" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
     </row>
     <row r="19" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
     </row>
     <row r="20" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
     </row>
     <row r="21" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
     </row>
     <row r="22" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
     </row>
     <row r="23" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
+      <c r="A23" s="11"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
     </row>
     <row r="24" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
+      <c r="A24" s="11"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
     </row>
     <row r="25" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
+      <c r="A25" s="11"/>
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
     </row>
     <row r="26" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9"/>
     <row r="27" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9"/>
     <row r="28" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
     </row>
     <row r="29" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
     </row>
     <row r="30" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
     </row>
     <row r="31" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
     </row>
     <row r="32" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A32" s="12"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
     </row>
     <row r="33" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
     </row>
     <row r="34" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A34" s="12"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
     </row>
     <row r="35" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A35" s="12"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
     </row>
     <row r="36" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A36" s="12"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
+      <c r="A36" s="7"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
     </row>
     <row r="37" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A37" s="12"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
     </row>
     <row r="38" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A38" s="12"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
+      <c r="A38" s="7"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
     </row>
     <row r="39" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A39" s="12"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
     </row>
     <row r="40" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A40" s="12"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
+      <c r="A40" s="7"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
     </row>
     <row r="41" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A41" s="12"/>
-      <c r="B41" s="12"/>
-      <c r="C41" s="12"/>
-      <c r="D41" s="12"/>
-      <c r="E41" s="12"/>
-      <c r="F41" s="12"/>
+      <c r="A41" s="7"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
     </row>
     <row r="42" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A42" s="12"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="12"/>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
-      <c r="F42" s="12"/>
+      <c r="A42" s="7"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
     </row>
     <row r="43" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A43" s="12"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
-      <c r="E43" s="12"/>
-      <c r="F43" s="12"/>
+      <c r="A43" s="7"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
     </row>
     <row r="44" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A44" s="12"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="12"/>
-      <c r="E44" s="12"/>
-      <c r="F44" s="12"/>
+      <c r="A44" s="7"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
     </row>
     <row r="45" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A45" s="12"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
-      <c r="E45" s="12"/>
-      <c r="F45" s="12"/>
+      <c r="A45" s="7"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
     </row>
     <row r="46" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A46" s="12"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="12"/>
-      <c r="D46" s="12"/>
-      <c r="E46" s="12"/>
-      <c r="F46" s="12"/>
+      <c r="A46" s="7"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
     </row>
     <row r="47" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A47" s="12"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="12"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="12"/>
+      <c r="A47" s="7"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
     </row>
     <row r="48" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A48" s="12"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="12"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="12"/>
+      <c r="A48" s="7"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
     </row>
     <row r="49" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A49" s="12"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="12"/>
-      <c r="D49" s="12"/>
-      <c r="E49" s="12"/>
-      <c r="F49" s="12"/>
+      <c r="A49" s="7"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
     </row>
     <row r="50" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A50" s="12"/>
-      <c r="B50" s="12"/>
-      <c r="C50" s="12"/>
-      <c r="D50" s="12"/>
-      <c r="E50" s="12"/>
-      <c r="F50" s="12"/>
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
     </row>
     <row r="51" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A51" s="12"/>
-      <c r="B51" s="12"/>
-      <c r="C51" s="12"/>
-      <c r="D51" s="12"/>
-      <c r="E51" s="12"/>
-      <c r="F51" s="12"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
     </row>
     <row r="52" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A52" s="12"/>
-      <c r="B52" s="12"/>
-      <c r="C52" s="12"/>
-      <c r="D52" s="12"/>
-      <c r="E52" s="12"/>
-      <c r="F52" s="12"/>
+      <c r="A52" s="7"/>
+      <c r="B52" s="7"/>
+      <c r="C52" s="7"/>
+      <c r="D52" s="7"/>
+      <c r="E52" s="7"/>
+      <c r="F52" s="7"/>
     </row>
     <row r="53" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A53" s="12"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="12"/>
-      <c r="D53" s="12"/>
-      <c r="E53" s="12"/>
-      <c r="F53" s="12"/>
+      <c r="A53" s="7"/>
+      <c r="B53" s="7"/>
+      <c r="C53" s="7"/>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7"/>
+      <c r="F53" s="7"/>
     </row>
     <row r="54" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A54" s="12"/>
-      <c r="B54" s="12"/>
-      <c r="C54" s="12"/>
-      <c r="D54" s="12"/>
-      <c r="E54" s="12"/>
-      <c r="F54" s="12"/>
+      <c r="A54" s="7"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="7"/>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7"/>
+      <c r="F54" s="7"/>
     </row>
     <row r="57" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A57" s="10" t="s">
+      <c r="A57" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
     </row>
     <row r="58" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
-      <c r="D58" s="11"/>
-      <c r="E58" s="11"/>
-      <c r="F58" s="11"/>
+      <c r="B58" s="6"/>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
     </row>
     <row r="59" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A59" s="11"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="11"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="11"/>
-      <c r="F59" s="11"/>
+      <c r="A59" s="6"/>
+      <c r="B59" s="6"/>
+      <c r="C59" s="6"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="6"/>
+      <c r="F59" s="6"/>
     </row>
     <row r="60" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A60" s="11"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="11"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="11"/>
-      <c r="F60" s="11"/>
+      <c r="A60" s="6"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
     </row>
     <row r="61" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A61" s="11"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="11"/>
-      <c r="F61" s="11"/>
+      <c r="A61" s="6"/>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="6"/>
     </row>
     <row r="62" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A62" s="11"/>
-      <c r="B62" s="11"/>
-      <c r="C62" s="11"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="11"/>
-      <c r="F62" s="11"/>
+      <c r="A62" s="6"/>
+      <c r="B62" s="6"/>
+      <c r="C62" s="6"/>
+      <c r="D62" s="6"/>
+      <c r="E62" s="6"/>
+      <c r="F62" s="6"/>
     </row>
     <row r="63" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A63" s="11"/>
-      <c r="B63" s="11"/>
-      <c r="C63" s="11"/>
-      <c r="D63" s="11"/>
-      <c r="E63" s="11"/>
-      <c r="F63" s="11"/>
+      <c r="A63" s="6"/>
+      <c r="B63" s="6"/>
+      <c r="C63" s="6"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="6"/>
+      <c r="F63" s="6"/>
     </row>
     <row r="64" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A64" s="11"/>
-      <c r="B64" s="11"/>
-      <c r="C64" s="11"/>
-      <c r="D64" s="11"/>
-      <c r="E64" s="11"/>
-      <c r="F64" s="11"/>
+      <c r="A64" s="6"/>
+      <c r="B64" s="6"/>
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
     </row>
     <row r="65" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A65" s="11"/>
-      <c r="B65" s="11"/>
-      <c r="C65" s="11"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="11"/>
-      <c r="F65" s="11"/>
+      <c r="A65" s="6"/>
+      <c r="B65" s="6"/>
+      <c r="C65" s="6"/>
+      <c r="D65" s="6"/>
+      <c r="E65" s="6"/>
+      <c r="F65" s="6"/>
     </row>
     <row r="66" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A66" s="11"/>
-      <c r="B66" s="11"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="11"/>
+      <c r="A66" s="6"/>
+      <c r="B66" s="6"/>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="6"/>
     </row>
     <row r="67" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A67" s="11"/>
-      <c r="B67" s="11"/>
-      <c r="C67" s="11"/>
-      <c r="D67" s="11"/>
-      <c r="E67" s="11"/>
-      <c r="F67" s="11"/>
+      <c r="A67" s="6"/>
+      <c r="B67" s="6"/>
+      <c r="C67" s="6"/>
+      <c r="D67" s="6"/>
+      <c r="E67" s="6"/>
+      <c r="F67" s="6"/>
     </row>
     <row r="68" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.9">
-      <c r="A68" s="11"/>
-      <c r="B68" s="11"/>
-      <c r="C68" s="11"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="11"/>
-      <c r="F68" s="11"/>
+      <c r="A68" s="6"/>
+      <c r="B68" s="6"/>
+      <c r="C68" s="6"/>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="6"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.9">
-      <c r="A69" s="11"/>
-      <c r="B69" s="11"/>
-      <c r="C69" s="11"/>
-      <c r="D69" s="11"/>
-      <c r="E69" s="11"/>
-      <c r="F69" s="11"/>
+      <c r="A69" s="6"/>
+      <c r="B69" s="6"/>
+      <c r="C69" s="6"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>